<commit_message>
update multiple files in data, outputs, and reports directories
</commit_message>
<xml_diff>
--- a/outputs/exports/data_powerpoint.xlsx
+++ b/outputs/exports/data_powerpoint.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Self Learning\data science projects\Hong Leong Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QS\datascience\HBA Capital\outputs\exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799939CA-EECD-4B5A-8E03-A2C2F8A060D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E5D2AC-5C86-4EB9-8E7E-AF6B13DBA0A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sum Assured by Product" sheetId="8" r:id="rId1"/>
@@ -27,9 +27,10 @@
     <pivotCache cacheId="0" r:id="rId9"/>
     <pivotCache cacheId="1" r:id="rId10"/>
     <pivotCache cacheId="2" r:id="rId11"/>
-    <pivotCache cacheId="21" r:id="rId12"/>
-    <pivotCache cacheId="26" r:id="rId13"/>
-    <pivotCache cacheId="31" r:id="rId14"/>
+    <pivotCache cacheId="3" r:id="rId12"/>
+    <pivotCache cacheId="4" r:id="rId13"/>
+    <pivotCache cacheId="6" r:id="rId14"/>
+    <pivotCache cacheId="21" r:id="rId15"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="192">
   <si>
     <t>Year</t>
   </si>
@@ -619,6 +620,15 @@
   <si>
     <t>With Premium Loss</t>
   </si>
+  <si>
+    <t>Active Policies</t>
+  </si>
+  <si>
+    <t>Policies Subscribed</t>
+  </si>
+  <si>
+    <t>Sum of Active Policies</t>
+  </si>
 </sst>
 </file>
 
@@ -681,13 +691,7 @@
   </cellStyles>
   <dxfs count="16">
     <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
+      <numFmt numFmtId="10" formatCode="&quot;RM&quot;#,##0;[Red]\-&quot;RM&quot;#,##0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
@@ -721,6 +725,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="12" formatCode="&quot;RM&quot;#,##0.00;[Red]\-&quot;RM&quot;#,##0.00"/>
@@ -1567,7 +1577,6 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1624,7 +1633,6 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1681,7 +1689,6 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1738,7 +1745,6 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1866,6 +1872,20 @@
             <c:idx val="3"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-03F2-4508-A12A-D6D6A4E7E6B3}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -2057,7 +2077,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -2466,6 +2485,230 @@
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
         <c:spPr>
           <a:solidFill>
             <a:schemeClr val="accent1"/>
@@ -3274,6 +3517,230 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -3286,7 +3753,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$G$41:$G$42</c:f>
+              <c:f>'Imbalance Segmentation'!$F$41:$F$42</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3307,7 +3774,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$F$43:$F$45</c:f>
+              <c:f>'Imbalance Segmentation'!$E$43:$E$45</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3321,15 +3788,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Imbalance Segmentation'!$G$43:$G$45</c:f>
+              <c:f>'Imbalance Segmentation'!$F$43:$F$45</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.30565448266715134</c:v>
+                  <c:v>0.18679127824051819</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.54238995962184933</c:v>
+                  <c:v>0.45730730387856261</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3345,7 +3812,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$H$41:$H$42</c:f>
+              <c:f>'Imbalance Segmentation'!$G$41:$G$42</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3366,7 +3833,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$F$43:$F$45</c:f>
+              <c:f>'Imbalance Segmentation'!$E$43:$E$45</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3380,15 +3847,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Imbalance Segmentation'!$H$43:$H$45</c:f>
+              <c:f>'Imbalance Segmentation'!$G$43:$G$45</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>3.7118134526680849E-2</c:v>
+                  <c:v>0.40168320186602152</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.509625293502848E-2</c:v>
+                  <c:v>0.32149021133094519</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3404,7 +3871,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$I$41:$I$42</c:f>
+              <c:f>'Imbalance Segmentation'!$H$41:$H$42</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3425,7 +3892,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$F$43:$F$45</c:f>
+              <c:f>'Imbalance Segmentation'!$E$43:$E$45</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3439,15 +3906,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Imbalance Segmentation'!$I$43:$I$45</c:f>
+              <c:f>'Imbalance Segmentation'!$H$43:$H$45</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.60481989261837277</c:v>
+                  <c:v>0.22515583013530233</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.38256417324198683</c:v>
+                  <c:v>0.10856041704879196</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3463,7 +3930,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$J$41:$J$42</c:f>
+              <c:f>'Imbalance Segmentation'!$I$41:$I$42</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3484,7 +3951,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Imbalance Segmentation'!$F$43:$F$45</c:f>
+              <c:f>'Imbalance Segmentation'!$E$43:$E$45</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3498,15 +3965,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Imbalance Segmentation'!$J$43:$J$45</c:f>
+              <c:f>'Imbalance Segmentation'!$I$43:$I$45</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>5.2407490187795044E-2</c:v>
+                  <c:v>0.18636968975815793</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.9949614201135353E-2</c:v>
+                  <c:v>0.11264206774170024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3634,6 +4101,761 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1129051152"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[data_powerpoint.xlsx]Imbalance Segmentation!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$G$55:$G$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Premium High, Coverage High</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$F$57:$F$61</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>A</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>D</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>E</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Imbalance Segmentation'!$G$57:$G$61</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.24320457796852646</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.22222222222222221</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.27142857142857141</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.25564218301189989</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C2B4-4247-8D0A-AE854297E1CA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$H$55:$H$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Premium High, Coverage Low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$F$57:$F$61</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>A</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>D</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>E</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Imbalance Segmentation'!$H$57:$H$61</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.25393419170243203</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.22222222222222221</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.22142857142857142</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.24661469019286009</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C2B4-4247-8D0A-AE854297E1CA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$I$55:$I$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Premium Low, Coverage High</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$F$57:$F$61</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>A</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>D</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>E</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Imbalance Segmentation'!$I$57:$I$61</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.25679542203147354</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.33333333333333331</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.22857142857142856</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.24907673368896183</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-C2B4-4247-8D0A-AE854297E1CA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$J$55:$J$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Premium Low, Coverage Low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Imbalance Segmentation'!$F$57:$F$61</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>A</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>D</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>E</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Imbalance Segmentation'!$J$57:$J$61</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.24606580829756797</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.22222222222222221</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.27857142857142858</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.24866639310627822</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-C2B4-4247-8D0A-AE854297E1CA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="75"/>
+        <c:overlap val="100"/>
+        <c:axId val="1915274768"/>
+        <c:axId val="1915275248"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1915274768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1915275248"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1915275248"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1915274768"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10917,6 +12139,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors13.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -12751,6 +14013,511 @@
 </file>
 
 <file path=xl/charts/style12.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style13.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -17779,6 +19546,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>485526</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>85600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>155863</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F1D91C5-0532-DA50-348C-20AD76F06ABF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18502,30 +20305,64 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="QS" refreshedDate="45503.924205671297" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{26B3EC96-32D5-4847-89AC-56135FE33C3F}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="QS" refreshedDate="45590.910039699076" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="16" xr:uid="{F6C38967-9333-4C01-A099-BAF6521BA257}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Table12"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="Insurance Product" numFmtId="0">
+      <sharedItems count="4">
+        <s v="A"/>
+        <s v="C"/>
+        <s v="D"/>
+        <s v="E"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Active Policies" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2" maxValue="623"/>
+    </cacheField>
+    <cacheField name="Imbalance Status by Insurance Product" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Premium High, Coverage High"/>
+        <s v="Premium High, Coverage Low"/>
+        <s v="Premium Low, Coverage High"/>
+        <s v="Premium Low, Coverage Low"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Median of Median Insured" numFmtId="8">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="85750" maxValue="3975000"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="QS" refreshedDate="45591.421646064817" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="8" xr:uid="{26B3EC96-32D5-4847-89AC-56135FE33C3F}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table9"/>
   </cacheSource>
-  <cacheFields count="4">
+  <cacheFields count="3">
     <cacheField name="Insurance Product" numFmtId="0">
       <sharedItems count="2">
+        <s v="A"/>
         <s v="E"/>
-        <s v="A"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Imbalance Status by Insurance Product" numFmtId="0">
       <sharedItems count="4">
         <s v="Premium High, Coverage High"/>
+        <s v="Premium High, Coverage Low"/>
         <s v="Premium Low, Coverage High"/>
         <s v="Premium Low, Coverage Low"/>
-        <s v="Premium High, Coverage Low"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Sum Assured" numFmtId="8">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="151125" maxValue="19866110"/>
-    </cacheField>
-    <cacheField name="Median of Median Insured" numFmtId="8">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="85750" maxValue="165000"/>
+    <cacheField name="Premium Loss" numFmtId="6">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="47301" maxValue="413875"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -21580,54 +23417,147 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="16">
+  <r>
+    <x v="0"/>
+    <n v="340"/>
+    <x v="0"/>
+    <n v="85750"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="355"/>
+    <x v="1"/>
+    <n v="85750"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="359"/>
+    <x v="2"/>
+    <n v="85750"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="344"/>
+    <x v="3"/>
+    <n v="85750"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="2"/>
+    <x v="0"/>
+    <n v="3975000"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="2"/>
+    <x v="1"/>
+    <n v="3975000"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="3"/>
+    <x v="2"/>
+    <n v="3975000"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="2"/>
+    <x v="3"/>
+    <n v="3975000"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="38"/>
+    <x v="0"/>
+    <n v="602870"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="31"/>
+    <x v="1"/>
+    <n v="602870"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="32"/>
+    <x v="2"/>
+    <n v="602870"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="39"/>
+    <x v="3"/>
+    <n v="602870"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="623"/>
+    <x v="0"/>
+    <n v="165000"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="601"/>
+    <x v="1"/>
+    <n v="165000"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="607"/>
+    <x v="2"/>
+    <n v="165000"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="606"/>
+    <x v="3"/>
+    <n v="165000"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="8">
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="19866110"/>
-    <n v="165000"/>
+    <n v="47408"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="14012173"/>
-    <n v="165000"/>
+    <n v="101948"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="57145"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="47301"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="413875"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
-    <n v="2462500"/>
-    <n v="85750"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="2"/>
-    <n v="1463234"/>
-    <n v="165000"/>
-  </r>
-  <r>
-    <x v="0"/>
-    <x v="3"/>
-    <n v="1285470"/>
-    <n v="165000"/>
-  </r>
-  <r>
-    <x v="1"/>
-    <x v="0"/>
-    <n v="1244460"/>
-    <n v="85750"/>
+    <n v="290957"/>
   </r>
   <r>
     <x v="1"/>
     <x v="2"/>
-    <n v="213375"/>
-    <n v="85750"/>
+    <n v="98250"/>
   </r>
   <r>
     <x v="1"/>
     <x v="3"/>
-    <n v="151125"/>
-    <n v="85750"/>
+    <n v="101944"/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -23036,247 +24966,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B9A2C35-2168-428A-BD64-A0A2BAE87644}" name="PivotTable14" cacheId="31" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="F41:K45" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="4">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" numFmtId="8" showAll="0"/>
-    <pivotField numFmtId="8" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" Sum Assured" fld="2" baseField="0" baseItem="0" numFmtId="10">
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{E15A36E0-9728-4e99-A89B-3F7291B0FE68}">
-          <x14:dataField pivotShowAs="percentOfParentCol"/>
-        </ext>
-      </extLst>
-    </dataField>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C038BBE2-6BFF-41BE-8A7B-16A9B3744A99}" name="PivotTable13" cacheId="26" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="F21:K27" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="4">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="1"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" numFmtId="8" showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="8" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" Premium Secured" fld="1" baseField="0" baseItem="2" numFmtId="10">
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{E15A36E0-9728-4e99-A89B-3F7291B0FE68}">
-          <x14:dataField pivotShowAs="percentOfParentCol"/>
-        </ext>
-      </extLst>
-    </dataField>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59122487-94C9-4E5D-BCCF-9118764B68B0}" name="PivotTable12" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59122487-94C9-4E5D-BCCF-9118764B68B0}" name="PivotTable12" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="F1:K7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
@@ -23477,12 +25167,423 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF1DCDB4-A17C-40C6-9356-C61AAE68D352}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+  <location ref="F55:K61" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="8" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Active Policies" fld="1" showDataAs="percentOfRow" baseField="0" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B9A2C35-2168-428A-BD64-A0A2BAE87644}" name="PivotTable14" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+  <location ref="E41:J45" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="6" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Premium Loss" fld="2" showDataAs="percentOfRow" baseField="0" baseItem="1" numFmtId="10"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C038BBE2-6BFF-41BE-8A7B-16A9B3744A99}" name="PivotTable13" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+  <location ref="F21:K27" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="8" showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="8" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name=" Premium Secured" fld="1" baseField="0" baseItem="2" numFmtId="10">
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{E15A36E0-9728-4e99-A89B-3F7291B0FE68}">
+          <x14:dataField pivotShowAs="percentOfParentCol"/>
+        </ext>
+      </extLst>
+    </dataField>
+  </dataFields>
+  <chartFormats count="8">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{3878F01A-1B61-47FE-9E82-A10E8C3ACB6B}" name="Table10" displayName="Table10" ref="A1:B5" totalsRowShown="0">
   <autoFilter ref="A1:B5" xr:uid="{3878F01A-1B61-47FE-9E82-A10E8C3ACB6B}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{8EA1896C-299D-4F63-BC63-E5E3FD911C8E}" name="Insurance Product"/>
-    <tableColumn id="2" xr3:uid="{DE625B63-D477-477B-91CF-5A3CFCAC256B}" name=" Sum Assured" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{DE625B63-D477-477B-91CF-5A3CFCAC256B}" name=" Sum Assured" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23493,22 +25594,34 @@
   <autoFilter ref="A21:D37" xr:uid="{6F98F0F5-7C7F-4A4B-9987-69A236733975}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B1B1D378-230E-4355-A1E3-CC23C83E78C3}" name="Insurance Product"/>
-    <tableColumn id="2" xr3:uid="{165B7CD0-9A0C-49E4-B433-9F997BA62C15}" name="Premium Secured" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{165B7CD0-9A0C-49E4-B433-9F997BA62C15}" name="Premium Secured" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{40CA2A3D-9B47-4A0C-BC25-F9CCCEE6633E}" name="Imbalance Status by Insurance Product"/>
-    <tableColumn id="4" xr3:uid="{AD22C415-B128-424D-BDBD-3B733084628B}" name="Average of Average Premiums" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{AD22C415-B128-424D-BDBD-3B733084628B}" name="Average of Average Premiums" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2929538F-6234-42B6-B2FA-35C543B9AA66}" name="Table9" displayName="Table9" ref="A41:D49" totalsRowShown="0">
-  <autoFilter ref="A41:D49" xr:uid="{2929538F-6234-42B6-B2FA-35C543B9AA66}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2929538F-6234-42B6-B2FA-35C543B9AA66}" name="Table9" displayName="Table9" ref="A41:C49" totalsRowShown="0">
+  <autoFilter ref="A41:C49" xr:uid="{2929538F-6234-42B6-B2FA-35C543B9AA66}"/>
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{83F5B694-D46A-49B1-A5EE-A407BD82450D}" name="Insurance Product"/>
     <tableColumn id="2" xr3:uid="{7128E6D7-1EF0-431D-8CBE-297036A9E2F9}" name="Imbalance Status by Insurance Product"/>
-    <tableColumn id="3" xr3:uid="{516D1444-DAFD-434E-83E3-7686600F25AD}" name="Sum Assured" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{13A64453-8CBF-4189-BC7A-F9BF852C4ECD}" name="Median of Median Insured" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{516D1444-DAFD-434E-83E3-7686600F25AD}" name="Premium Loss" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{9E51D493-8435-478A-A974-BA2E1AE5F794}" name="Table12" displayName="Table12" ref="A55:D71" totalsRowShown="0">
+  <autoFilter ref="A55:D71" xr:uid="{9E51D493-8435-478A-A974-BA2E1AE5F794}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{523074A8-D211-4A56-B1B7-B6989301F197}" name="Insurance Product"/>
+    <tableColumn id="2" xr3:uid="{18582873-E478-4679-BBF2-6846682FCD57}" name="Active Policies"/>
+    <tableColumn id="3" xr3:uid="{D0C51040-F363-440D-822F-273D8967786C}" name="Imbalance Status by Insurance Product"/>
+    <tableColumn id="4" xr3:uid="{9D450C90-7AA8-4F38-9A44-6FA3E30EF09F}" name="Median of Median Insured" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23519,7 +25632,7 @@
   <autoFilter ref="A1:B5" xr:uid="{327AFAB1-D047-4375-B1C1-2A9EEBAFE0B4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C08F3612-E357-4928-9285-EA7C79637C6F}" name="Insurance Product"/>
-    <tableColumn id="2" xr3:uid="{8AA004A0-B110-4D12-AC18-7BEE05FE4537}" name="Premium Secured" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{8AA004A0-B110-4D12-AC18-7BEE05FE4537}" name="Premium Secured" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23532,7 +25645,7 @@
     <tableColumn id="1" xr3:uid="{75191D2D-E05D-41C4-BB03-77A261B5B491}" name="Year"/>
     <tableColumn id="2" xr3:uid="{DBA72B23-3A8F-4917-AED1-6021239FEF5B}" name="Month"/>
     <tableColumn id="3" xr3:uid="{32FF73DF-45FC-47E9-A5CF-7894EB696F24}" name="Day"/>
-    <tableColumn id="4" xr3:uid="{39A59DF3-6C95-480A-B8D0-AAD920A0BC35}" name="Premium Secured" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{39A59DF3-6C95-480A-B8D0-AAD920A0BC35}" name="Premium Secured" dataDxfId="13"/>
     <tableColumn id="5" xr3:uid="{2D7EFA25-D277-4676-8161-FD3F368DD372}" name="Premium Loss"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -23544,7 +25657,7 @@
   <autoFilter ref="G41:I45" xr:uid="{B6189DED-1B3A-4457-801F-CEF786B21D50}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{CCA8A1C5-5465-4BFD-8A38-BBB46F0324B8}" name="Insurance Product"/>
-    <tableColumn id="2" xr3:uid="{5AC01660-2626-4F0E-96FB-519DA0CA2C39}" name="Premium Earned" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{5AC01660-2626-4F0E-96FB-519DA0CA2C39}" name="Premium Earned" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{2032F2DB-18D0-44FE-81D4-38D2CD8EC87A}" name="Premium Loss"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -23555,9 +25668,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{64F3B7B5-30D3-4510-A827-DEA418642AD5}" name="Table2" displayName="Table2" ref="A1:C361" totalsRowShown="0">
   <autoFilter ref="A1:C361" xr:uid="{64F3B7B5-30D3-4510-A827-DEA418642AD5}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BAFE58F3-4847-497A-92D8-1A7AE75EC1C3}" name="Date Issued" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{BAFE58F3-4847-497A-92D8-1A7AE75EC1C3}" name="Date Issued" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{6F93BC29-129F-46A8-AAF6-DD95A413CBC8}" name="Insurance Product"/>
-    <tableColumn id="3" xr3:uid="{0EA7CBD4-A711-4080-8668-5C710606A188}" name="Premium Earned" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{0EA7CBD4-A711-4080-8668-5C710606A188}" name="Premium Earned" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23569,7 +25682,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{236CCB13-8C59-40B9-BDD8-A3074F4F293B}" name="Imbalances"/>
     <tableColumn id="2" xr3:uid="{D0D474CA-D2F0-49C8-9DC4-527DC6E0BD50}" name="Clients Count"/>
-    <tableColumn id="3" xr3:uid="{68BDEBB2-9E47-40D9-B146-834126324520}" name="Premiums Charged" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{68BDEBB2-9E47-40D9-B146-834126324520}" name="Premiums Charged" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23580,9 +25693,9 @@
   <autoFilter ref="A1:D5" xr:uid="{7B015126-618F-4849-899F-1335406018C9}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DF765A87-DE7C-44F7-9262-EBAD60C8261F}" name="Insurance Product"/>
-    <tableColumn id="2" xr3:uid="{D4285844-8F5E-43F1-B76B-39E08B54B43B}" name=" Median Sum Assured Per Plan" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{3775B8D9-DEDB-45E3-881F-537DE5381FC5}" name="Average Premium Secured Per Plan" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{3985F30B-2B4F-4DF2-845F-3B091D77C888}" name="Ratio" dataDxfId="8">
+    <tableColumn id="2" xr3:uid="{D4285844-8F5E-43F1-B76B-39E08B54B43B}" name=" Median Sum Assured Per Plan" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{3775B8D9-DEDB-45E3-881F-537DE5381FC5}" name="Average Premium Secured Per Plan" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{3985F30B-2B4F-4DF2-845F-3B091D77C888}" name="Ratio" dataDxfId="6">
       <calculatedColumnFormula>ROUND(Table16[[#This Row],[ Median Sum Assured Per Plan]]/Table16[[#This Row],[Average Premium Secured Per Plan]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -23608,8 +25721,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{206E08FC-87A3-49A2-83E8-F92588A2F95A}" name="Insurance Product"/>
     <tableColumn id="2" xr3:uid="{A5909B18-67BF-4A7F-8156-5EE57CB61D27}" name="Imbalance Status by Insurance Product"/>
-    <tableColumn id="3" xr3:uid="{C4B55F54-DB93-40F0-9F7E-D4A9B40FAE84}" name="Sum Assured" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{8D6F8E0B-3806-4B67-8D4F-6374D4A34694}" name="Median of Median Insured" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{C4B55F54-DB93-40F0-9F7E-D4A9B40FAE84}" name="Sum Assured" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{8D6F8E0B-3806-4B67-8D4F-6374D4A34694}" name="Median of Median Insured" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -33019,17 +35132,17 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDE55C5D-6128-45E7-BDE8-FC089B1392D1}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="3" width="37" customWidth="1"/>
     <col min="4" max="4" width="29.85546875" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="15" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="31.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -33671,7 +35784,7 @@
         <v>2060.44</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -33685,7 +35798,7 @@
         <v>2060.44</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -33699,7 +35812,7 @@
         <v>2060.44</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -33713,7 +35826,7 @@
         <v>2060.44</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -33727,7 +35840,7 @@
         <v>1559.41</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -33741,12 +35854,12 @@
         <v>1559.41</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>10</v>
       </c>
@@ -33754,209 +35867,540 @@
         <v>182</v>
       </c>
       <c r="C41" t="s">
-        <v>184</v>
-      </c>
-      <c r="D41" t="s">
-        <v>185</v>
+        <v>4</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="G41" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B42" t="s">
         <v>162</v>
       </c>
-      <c r="C42" s="1">
-        <v>19866110</v>
-      </c>
-      <c r="D42" s="1">
-        <v>165000</v>
-      </c>
-      <c r="F42" s="3" t="s">
+      <c r="C42" s="2">
+        <v>47408</v>
+      </c>
+      <c r="E42" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="F42" t="s">
+        <v>162</v>
+      </c>
       <c r="G42" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H42" t="s">
+        <v>167</v>
+      </c>
+      <c r="I42" t="s">
+        <v>163</v>
+      </c>
+      <c r="J42" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" t="s">
         <v>166</v>
       </c>
-      <c r="I42" t="s">
-        <v>167</v>
-      </c>
-      <c r="J42" t="s">
-        <v>163</v>
-      </c>
-      <c r="K42" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>15</v>
-      </c>
-      <c r="B43" t="s">
-        <v>167</v>
-      </c>
-      <c r="C43" s="1">
-        <v>14012173</v>
-      </c>
-      <c r="D43" s="1">
-        <v>165000</v>
-      </c>
-      <c r="F43" s="4" t="s">
+      <c r="C43" s="2">
+        <v>101948</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="F43" s="10">
+        <v>0.18679127824051819</v>
+      </c>
       <c r="G43" s="10">
-        <v>0.30565448266715134</v>
+        <v>0.40168320186602152</v>
       </c>
       <c r="H43" s="10">
-        <v>3.7118134526680849E-2</v>
+        <v>0.22515583013530233</v>
       </c>
       <c r="I43" s="10">
-        <v>0.60481989261837277</v>
+        <v>0.18636968975815793</v>
       </c>
       <c r="J43" s="10">
-        <v>5.2407490187795044E-2</v>
-      </c>
-      <c r="K43" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>12</v>
       </c>
       <c r="B44" t="s">
         <v>167</v>
       </c>
-      <c r="C44" s="1">
-        <v>2462500</v>
-      </c>
-      <c r="D44" s="1">
-        <v>85750</v>
-      </c>
-      <c r="F44" s="4" t="s">
+      <c r="C44" s="2">
+        <v>57145</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="F44" s="10">
+        <v>0.45730730387856261</v>
+      </c>
       <c r="G44" s="10">
-        <v>0.54238995962184933</v>
+        <v>0.32149021133094519</v>
       </c>
       <c r="H44" s="10">
-        <v>3.509625293502848E-2</v>
+        <v>0.10856041704879196</v>
       </c>
       <c r="I44" s="10">
-        <v>0.38256417324198683</v>
+        <v>0.11264206774170024</v>
       </c>
       <c r="J44" s="10">
-        <v>3.9949614201135353E-2</v>
-      </c>
-      <c r="K44" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B45" t="s">
         <v>163</v>
       </c>
-      <c r="C45" s="1">
-        <v>1463234</v>
-      </c>
-      <c r="D45" s="1">
-        <v>165000</v>
-      </c>
-      <c r="F45" s="4" t="s">
+      <c r="C45" s="2">
+        <v>47301</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="F45" s="10">
+        <v>0.39805993641851939</v>
+      </c>
       <c r="G45" s="10">
-        <v>0.51870701601955471</v>
+        <v>0.33905376811744281</v>
       </c>
       <c r="H45" s="10">
-        <v>3.5298521341612862E-2</v>
+        <v>0.13409669079449238</v>
       </c>
       <c r="I45" s="10">
-        <v>0.40479856639247191</v>
+        <v>0.12878960466954545</v>
       </c>
       <c r="J45" s="10">
-        <v>4.1195896246360456E-2</v>
-      </c>
-      <c r="K45" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>15</v>
       </c>
       <c r="B46" t="s">
+        <v>162</v>
+      </c>
+      <c r="C46" s="2">
+        <v>413875</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" t="s">
         <v>166</v>
       </c>
-      <c r="C46" s="1">
-        <v>1285470</v>
-      </c>
-      <c r="D46" s="1">
+      <c r="C47" s="2">
+        <v>290957</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" t="s">
+        <v>167</v>
+      </c>
+      <c r="C48" s="2">
+        <v>98250</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" t="s">
+        <v>163</v>
+      </c>
+      <c r="C49" s="2">
+        <v>101944</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>10</v>
+      </c>
+      <c r="B55" t="s">
+        <v>189</v>
+      </c>
+      <c r="C55" t="s">
+        <v>182</v>
+      </c>
+      <c r="D55" t="s">
+        <v>185</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56">
+        <v>340</v>
+      </c>
+      <c r="C56" t="s">
+        <v>162</v>
+      </c>
+      <c r="D56" s="1">
+        <v>85750</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G56" t="s">
+        <v>162</v>
+      </c>
+      <c r="H56" t="s">
+        <v>166</v>
+      </c>
+      <c r="I56" t="s">
+        <v>167</v>
+      </c>
+      <c r="J56" t="s">
+        <v>163</v>
+      </c>
+      <c r="K56" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57">
+        <v>355</v>
+      </c>
+      <c r="C57" t="s">
+        <v>166</v>
+      </c>
+      <c r="D57" s="1">
+        <v>85750</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" s="10">
+        <v>0.24320457796852646</v>
+      </c>
+      <c r="H57" s="10">
+        <v>0.25393419170243203</v>
+      </c>
+      <c r="I57" s="10">
+        <v>0.25679542203147354</v>
+      </c>
+      <c r="J57" s="10">
+        <v>0.24606580829756797</v>
+      </c>
+      <c r="K57" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58">
+        <v>359</v>
+      </c>
+      <c r="C58" t="s">
+        <v>167</v>
+      </c>
+      <c r="D58" s="1">
+        <v>85750</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="10">
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="H58" s="10">
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="I58" s="10">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="J58" s="10">
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="K58" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59">
+        <v>344</v>
+      </c>
+      <c r="C59" t="s">
+        <v>163</v>
+      </c>
+      <c r="D59" s="1">
+        <v>85750</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" s="10">
+        <v>0.27142857142857141</v>
+      </c>
+      <c r="H59" s="10">
+        <v>0.22142857142857142</v>
+      </c>
+      <c r="I59" s="10">
+        <v>0.22857142857142856</v>
+      </c>
+      <c r="J59" s="10">
+        <v>0.27857142857142858</v>
+      </c>
+      <c r="K59" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60">
+        <v>2</v>
+      </c>
+      <c r="C60" t="s">
+        <v>162</v>
+      </c>
+      <c r="D60" s="1">
+        <v>3975000</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G60" s="10">
+        <v>0.25564218301189989</v>
+      </c>
+      <c r="H60" s="10">
+        <v>0.24661469019286009</v>
+      </c>
+      <c r="I60" s="10">
+        <v>0.24907673368896183</v>
+      </c>
+      <c r="J60" s="10">
+        <v>0.24866639310627822</v>
+      </c>
+      <c r="K60" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61" t="s">
+        <v>166</v>
+      </c>
+      <c r="D61" s="1">
+        <v>3975000</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G61" s="10">
+        <v>0.25175702811244982</v>
+      </c>
+      <c r="H61" s="10">
+        <v>0.24824297188755021</v>
+      </c>
+      <c r="I61" s="10">
+        <v>0.2512550200803213</v>
+      </c>
+      <c r="J61" s="10">
+        <v>0.24874497991967873</v>
+      </c>
+      <c r="K61" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>167</v>
+      </c>
+      <c r="D62" s="1">
+        <v>3975000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63" t="s">
+        <v>163</v>
+      </c>
+      <c r="D63" s="1">
+        <v>3975000</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64">
+        <v>38</v>
+      </c>
+      <c r="C64" t="s">
+        <v>162</v>
+      </c>
+      <c r="D64" s="1">
+        <v>602870</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>14</v>
+      </c>
+      <c r="B65">
+        <v>31</v>
+      </c>
+      <c r="C65" t="s">
+        <v>166</v>
+      </c>
+      <c r="D65" s="1">
+        <v>602870</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>14</v>
+      </c>
+      <c r="B66">
+        <v>32</v>
+      </c>
+      <c r="C66" t="s">
+        <v>167</v>
+      </c>
+      <c r="D66" s="1">
+        <v>602870</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>14</v>
+      </c>
+      <c r="B67">
+        <v>39</v>
+      </c>
+      <c r="C67" t="s">
+        <v>163</v>
+      </c>
+      <c r="D67" s="1">
+        <v>602870</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>15</v>
+      </c>
+      <c r="B68">
+        <v>623</v>
+      </c>
+      <c r="C68" t="s">
+        <v>162</v>
+      </c>
+      <c r="D68" s="1">
         <v>165000</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>12</v>
-      </c>
-      <c r="B47" t="s">
-        <v>162</v>
-      </c>
-      <c r="C47" s="1">
-        <v>1244460</v>
-      </c>
-      <c r="D47" s="1">
-        <v>85750</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>15</v>
+      </c>
+      <c r="B69">
+        <v>601</v>
+      </c>
+      <c r="C69" t="s">
+        <v>166</v>
+      </c>
+      <c r="D69" s="1">
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>15</v>
+      </c>
+      <c r="B70">
+        <v>607</v>
+      </c>
+      <c r="C70" t="s">
+        <v>167</v>
+      </c>
+      <c r="D70" s="1">
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>15</v>
+      </c>
+      <c r="B71">
+        <v>606</v>
+      </c>
+      <c r="C71" t="s">
         <v>163</v>
       </c>
-      <c r="C48" s="1">
-        <v>213375</v>
-      </c>
-      <c r="D48" s="1">
-        <v>85750</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" t="s">
-        <v>166</v>
-      </c>
-      <c r="C49" s="1">
-        <v>151125</v>
-      </c>
-      <c r="D49" s="1">
-        <v>85750</v>
+      <c r="D71" s="1">
+        <v>165000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
-  <tableParts count="3">
-    <tablePart r:id="rId5"/>
+  <drawing r:id="rId5"/>
+  <tableParts count="4">
     <tablePart r:id="rId6"/>
     <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>